<commit_message>
Removidos dados com erros do arquivo erros.ipynb
</commit_message>
<xml_diff>
--- a/output_data_cnae/cnpj_limpos_.xlsx
+++ b/output_data_cnae/cnpj_limpos_.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -945,6 +945,476 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07.589.579/0001-19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>JJ ANALIA FAST FOOD LTDA.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>diretoria@griletto.com.br</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589579000119</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5611-2/03</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Lanchonetes, casas de chá, de sucos e similares</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:30:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07.589.683/0001-03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>VBX CORRETORA DE SEGUROS LTDA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Niterói</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ederwil@bol.com.br</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589683000103</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6622-3/00</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Corretores e agentes de seguros, de planos de previdência complementar e de saúde</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:31:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07.589.745/0001-87</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AGROTERRA PRODUTOS AGROPECUARIOS LTDA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ituporanga</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>e-mail não cadastrado</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589745000187</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4683-4/00</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Comércio atacadista de defensivos agrícolas, adubos, fertilizantes e corretivos do solo</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:31:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07.589.867/0001-73</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ALGOMIX AGROINDUSTRIAL LTDA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ouro Verde do Oeste</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>davi@algomix.com.br</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589867000173</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1066-0/00</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Fabricação de alimentos para animais</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:31:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07.589.892/0001-57</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AQUILAE DO JARDIM LTDA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>jardim@redeaquilae.com.br</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589892000157</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4731-8/00</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Comércio varejista de combustíveis para veículos automotores</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:32:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07.589.967/0001-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CLAMA- COMERCIO DE MATERIAIS DE CONSTRUCAO LTDA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>clamatec@hotmail.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07589967000108</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4744-0/99</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Comércio varejista de materiais de construção em geral</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:32:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07.590.039/0001-55</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CICERA DO SOCORRO DOS SANTOS BALBINO</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Remígio</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>e-mail não cadastrado</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07590039000155</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4731-8/00</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Comércio varejista de combustíveis para veículos automotores</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:32:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07.590.106/0001-31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VIXRAX PARTICIPACOES LTDA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>carlos.serafini@solucont.com.br</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07590106000131</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6462-0/00</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Holdings de instituições não financeiras</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:33:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07.590.116/0001-77</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ITAPEMIRIM RENOVADORA E COMERCIO DE PNEUS LTDA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cachoeiro de Itapemirim</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>itapemirim.renovadora@gmail.com</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07590116000177</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2212-9/00</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Reforma de pneumáticos usados</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:33:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07.590.448/0001-51</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ASTENJOHNSON DO BRASIL EQUIPAMENTOS PARA INDUSTRIA DE PAPEL, CELULOSE E NAO-TECIDOS LTDA.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Nova Odessa</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>marcelo.munhoz@astenjohnson.com</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://cnpj.biz/07590448000151</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4663-0/00</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Comércio atacadista de máquinas e equipamentos para uso industrial; partes e peças</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2025-08-06 16:33:54</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>